<commit_message>
10.0 add Guide feature
</commit_message>
<xml_diff>
--- a/Repository/Settings/Translations.xlsx
+++ b/Repository/Settings/Translations.xlsx
@@ -929,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D483"/>
+  <dimension ref="A1:D486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9158,6 +9158,57 @@
         </is>
       </c>
     </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Information</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Messages</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Show/Hide Guide</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Afficher/Cacher le guide</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:D503"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>